<commit_message>
Updated weights for sensitivity analysis
Based on new GBD data on risk-factor contributions to DALYs 2023
</commit_message>
<xml_diff>
--- a/tables/Supp_Tables_PHI-SensAnalyse.xlsx
+++ b/tables/Supp_Tables_PHI-SensAnalyse.xlsx
@@ -431,7 +431,7 @@
         <v>24</v>
       </c>
       <c r="D2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -445,7 +445,7 @@
         <v>36</v>
       </c>
       <c r="D3" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4">
@@ -473,7 +473,7 @@
         <v>33</v>
       </c>
       <c r="D5" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         <v>37</v>
       </c>
       <c r="D6" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -501,7 +501,7 @@
         <v>62</v>
       </c>
       <c r="D7" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8">
@@ -529,7 +529,7 @@
         <v>22</v>
       </c>
       <c r="D9" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -543,7 +543,7 @@
         <v>57</v>
       </c>
       <c r="D10" t="n">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11">
@@ -557,7 +557,7 @@
         <v>47</v>
       </c>
       <c r="D11" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12">
@@ -571,7 +571,7 @@
         <v>49</v>
       </c>
       <c r="D12" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13">
@@ -585,7 +585,7 @@
         <v>22</v>
       </c>
       <c r="D13" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14">
@@ -599,7 +599,7 @@
         <v>38</v>
       </c>
       <c r="D14" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -613,7 +613,7 @@
         <v>55</v>
       </c>
       <c r="D15" t="n">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16">
@@ -627,7 +627,7 @@
         <v>49</v>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17">
@@ -641,7 +641,7 @@
         <v>49</v>
       </c>
       <c r="D17" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18">
@@ -655,7 +655,7 @@
         <v>22</v>
       </c>
       <c r="D18" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19">
@@ -669,7 +669,7 @@
         <v>64</v>
       </c>
       <c r="D19" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>